<commit_message>
n8n board refresh 2026-06-12T17:47:51Z
</commit_message>
<xml_diff>
--- a/app/reports/ARDT_research.xlsx
+++ b/app/reports/ARDT_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-11 17:40 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-12 17:40 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>9.5601</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04527999877929687</v>
+        <v>0.04479000091552734</v>
       </c>
     </row>
     <row r="6">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>143350025.2089413</v>
+        <v>143350030.8994709</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>9.5601</v>
+        <v>9.449999999999999</v>
       </c>
     </row>
     <row r="38">
@@ -1508,16 +1508,16 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>1370440576</v>
+        <v>1354657792</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>10.06</v>
+        <v>10.05</v>
       </c>
       <c r="E5" s="31" t="n">
-        <v>6.79</v>
+        <v>6.89</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>0.53</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="6">
@@ -1532,14 +1532,14 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>2301934592</v>
+        <v>2312970496</v>
       </c>
       <c r="D6" s="33" t="n"/>
       <c r="E6" s="33" t="n">
-        <v>8.407</v>
+        <v>8.561</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>1.466</v>
+        <v>1.493</v>
       </c>
     </row>
     <row r="7">
@@ -1554,16 +1554,16 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>1734517632</v>
+        <v>1757568640</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>17.145756</v>
+        <v>17.373615</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>10.879</v>
+        <v>10.864</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>1.201</v>
+        <v>1.199</v>
       </c>
     </row>
     <row r="8">
@@ -1578,16 +1578,16 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>1969701120</v>
+        <v>1952505728</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>65.12295</v>
+        <v>64.55443</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>14.311</v>
+        <v>14.659</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>0.648</v>
+        <v>0.664</v>
       </c>
     </row>
     <row r="9">
@@ -1602,16 +1602,16 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>1542795648</v>
+        <v>1535174144</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>5.855372</v>
+        <v>5.826446</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>9.048</v>
+        <v>9.125</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>1.112</v>
+        <v>1.122</v>
       </c>
     </row>
     <row r="10">
@@ -1626,14 +1626,14 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>3157183488</v>
+        <v>3155989504</v>
       </c>
       <c r="D10" s="33" t="n"/>
       <c r="E10" s="33" t="n">
-        <v>18.035</v>
+        <v>17.953</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>2.79</v>
+        <v>2.777</v>
       </c>
     </row>
     <row r="11">
@@ -1648,14 +1648,14 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>7525238272</v>
+        <v>7420503040</v>
       </c>
       <c r="D11" s="33" t="n"/>
       <c r="E11" s="33" t="n">
-        <v>-32.823</v>
+        <v>-33.762</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>57.138</v>
+        <v>58.772</v>
       </c>
     </row>
     <row r="12">
@@ -1670,16 +1670,16 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>3178771456</v>
+        <v>3243683584</v>
       </c>
       <c r="D12" s="33" t="n">
-        <v>138.75</v>
+        <v>141.58333</v>
       </c>
       <c r="E12" s="33" t="n">
-        <v>33.221</v>
+        <v>36.123</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>2.228</v>
+        <v>2.423</v>
       </c>
     </row>
     <row r="13">
@@ -1694,16 +1694,16 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>1983244160</v>
+        <v>1988992640</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v>11.723301</v>
+        <v>11.757281</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>8.372</v>
+        <v>8.555999999999999</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>1.134</v>
+        <v>1.159</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-06-13T17:47:03Z
</commit_message>
<xml_diff>
--- a/app/reports/ARDT_research.xlsx
+++ b/app/reports/ARDT_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-12 17:40 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-13 17:40 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>9.449999999999999</v>
+        <v>9.35</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04479000091552734</v>
+        <v>0.04486999988555909</v>
       </c>
     </row>
     <row r="6">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>143350030.8994709</v>
+        <v>143350033.7967915</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>9.449999999999999</v>
+        <v>9.35</v>
       </c>
     </row>
     <row r="38">
@@ -1508,16 +1508,16 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>1354657792</v>
+        <v>1340322816</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>10.05</v>
+        <v>9.84</v>
       </c>
       <c r="E5" s="31" t="n">
-        <v>6.89</v>
+        <v>6.8</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>0.54</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="6">
@@ -1532,14 +1532,14 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>2312970496</v>
+        <v>2262388736</v>
       </c>
       <c r="D6" s="33" t="n"/>
       <c r="E6" s="33" t="n">
-        <v>8.561</v>
+        <v>8.515000000000001</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>1.493</v>
+        <v>1.485</v>
       </c>
     </row>
     <row r="7">
@@ -1554,16 +1554,16 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>1757568640</v>
+        <v>1741050240</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>17.373615</v>
+        <v>17.210331</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>10.864</v>
+        <v>10.891</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>1.199</v>
+        <v>1.202</v>
       </c>
     </row>
     <row r="8">
@@ -1578,16 +1578,16 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>1952505728</v>
+        <v>1914911488</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>64.55443</v>
+        <v>63.311474</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>14.659</v>
+        <v>14.277</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>0.664</v>
+        <v>0.646</v>
       </c>
     </row>
     <row r="9">
@@ -1602,16 +1602,16 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>1535174144</v>
+        <v>1543884416</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>5.826446</v>
+        <v>5.859504</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>9.125</v>
+        <v>9.188000000000001</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>1.122</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="10">
@@ -1626,14 +1626,14 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>3155989504</v>
+        <v>3207335424</v>
       </c>
       <c r="D10" s="33" t="n"/>
       <c r="E10" s="33" t="n">
-        <v>17.953</v>
+        <v>18.205</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>2.777</v>
+        <v>2.816</v>
       </c>
     </row>
     <row r="11">
@@ -1648,14 +1648,14 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>7420503040</v>
+        <v>7436213248</v>
       </c>
       <c r="D11" s="33" t="n"/>
       <c r="E11" s="33" t="n">
-        <v>-33.762</v>
+        <v>-33.335</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>58.772</v>
+        <v>58.029</v>
       </c>
     </row>
     <row r="12">
@@ -1670,16 +1670,16 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>3243683584</v>
+        <v>3245592576</v>
       </c>
       <c r="D12" s="33" t="n">
-        <v>141.58333</v>
+        <v>141.66667</v>
       </c>
       <c r="E12" s="33" t="n">
-        <v>36.123</v>
+        <v>35.697</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>2.423</v>
+        <v>2.394</v>
       </c>
     </row>
     <row r="13">
@@ -1694,16 +1694,16 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>1988992640</v>
+        <v>1995562368</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v>11.757281</v>
+        <v>11.796117</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>8.555999999999999</v>
+        <v>8.599</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>1.159</v>
+        <v>1.164</v>
       </c>
     </row>
     <row r="15">

</xml_diff>